<commit_message>
now with ODB++ output added
</commit_message>
<xml_diff>
--- a/manufacturing/BOM/BOM_AFC_v4.0.2_DUNE.xlsx
+++ b/manufacturing/BOM/BOM_AFC_v4.0.2_DUNE.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://imperiallondon-my.sharepoint.com/personal/dparker_ic_ac_uk/Documents/Desktop/DUNE-Variant-AMC-FMC-Carrier-AFC/manufacturing/BOM/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{50100653-A88B-4831-8177-A1091D146525}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{D7426976-4EF7-480E-8FC6-5A914252A453}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="780" yWindow="780" windowWidth="21600" windowHeight="12525" xr2:uid="{08F11166-278B-45BC-B5A5-6E99F0561136}"/>
+    <workbookView xWindow="780" yWindow="780" windowWidth="21600" windowHeight="12525" xr2:uid="{CE486198-504E-485A-A6E7-F3D9F863E874}"/>
   </bookViews>
   <sheets>
     <sheet name="BOM_AFC_v4.0.2_DUNE" sheetId="1" r:id="rId1"/>
@@ -2180,7 +2180,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2D6F4478-7259-49B6-9A60-7F33D82ED197}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{730E29D2-F51B-4DE6-A630-B11EDAB21D6F}">
   <dimension ref="A1:I142"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>

</xml_diff>

<commit_message>
Output updated to reflect fit options
</commit_message>
<xml_diff>
--- a/manufacturing/BOM/BOM_AFC_v4.0.2_DUNE.xlsx
+++ b/manufacturing/BOM/BOM_AFC_v4.0.2_DUNE.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://imperiallondon-my.sharepoint.com/personal/dparker_ic_ac_uk/Documents/Desktop/DUNE-Variant-AMC-FMC-Carrier-AFC/manufacturing/BOM/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D7426976-4EF7-480E-8FC6-5A914252A453}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{EAD7384D-BA8E-4A7A-89A7-296925E9A63C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="780" yWindow="780" windowWidth="21600" windowHeight="12525" xr2:uid="{CE486198-504E-485A-A6E7-F3D9F863E874}"/>
+    <workbookView xWindow="780" yWindow="780" windowWidth="21600" windowHeight="12525" xr2:uid="{8008DD11-5676-44FF-B18F-B43FD6128FEF}"/>
   </bookViews>
   <sheets>
     <sheet name="BOM_AFC_v4.0.2_DUNE" sheetId="1" r:id="rId1"/>
@@ -2180,7 +2180,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{730E29D2-F51B-4DE6-A630-B11EDAB21D6F}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{90DCCCAB-9FDB-4AB7-BF6D-35D1459FC317}">
   <dimension ref="A1:I142"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>

</xml_diff>